<commit_message>
feat: add Existing Service Name dropdown to intake template (Item #23 §2.4)
Excel data validation on Overview!C13, listing the three current
services/<n>/ folders (REQ-2026-01/02/03), as defense-in-depth for
BA-entry typos alongside (not instead of) implementation_coordinator.py's
Layer 2 raise-on-mismatch backstop. Static list -- needs manual upkeep
as new services ship; the Layer 2 backstop covers drift.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Intake Template.xlsx
+++ b/docs/Intake Template.xlsx
@@ -1102,6 +1102,11 @@
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A16:C16"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="C13" showDropDown="0" showInputMessage="1" showErrorMessage="0" allowBlank="1" promptTitle="Existing Service Name" prompt="Pick the exact services/&lt;name&gt;/ folder this Enhancement targets. If it's not listed (a newer service), type the exact folder name manually -- this list needs manual upkeep as new services ship." type="list">
+      <formula1>"REQ-2026-01,REQ-2026-02,REQ-2026-03"</formula1>
+    </dataValidation>
+  </dataValidations>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>